<commit_message>
fix: update line_id mapping for 1004 and fix TRAIN_MONTHS reference
- Update line_id_2025.xlsx with Novomykolaivka mapped to 1004
- Fix regression_lines code: replace removed TRAIN_MONTHS with
  date-based TRAIN_START/TRAIN_END filtering

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/line_id_2025.xlsx
+++ b/backend/data/line_id_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HL\HLViewer\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEB9DAD-7852-4BD7-8F52-F4F832672037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC6F51D-0A41-4F9F-A69F-624404646958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="line_id" sheetId="1" r:id="rId1"/>
@@ -301,7 +301,7 @@
         <v>0</v>
       </c>
       <c r="B7">
-        <v>15</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>